<commit_message>
docs & tests: update user E2E test credentials and add generated report
</commit_message>
<xml_diff>
--- a/tests/ev_test_report.xlsx
+++ b/tests/ev_test_report.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-06-13 13:42:08</t>
+          <t>2026-06-16 21:19:10</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>prabha.testuser@example.com</t>
+          <t>prabha02102005@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>html_len=93765</t>
+          <t>html_len=93759</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
@@ -1019,7 +1019,7 @@
       <c r="I2" s="9" t="inlineStr"/>
       <c r="J2" s="9" t="inlineStr">
         <is>
-          <t>13:30:40</t>
+          <t>21:07:41</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       <c r="I3" s="11" t="inlineStr"/>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>13:30:43</t>
+          <t>21:07:44</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1115,7 @@
       <c r="I4" s="9" t="inlineStr"/>
       <c r="J4" s="9" t="inlineStr">
         <is>
-          <t>13:30:49</t>
+          <t>21:07:50</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       <c r="I5" s="11" t="inlineStr"/>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>13:30:56</t>
+          <t>21:07:56</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       <c r="I6" s="9" t="inlineStr"/>
       <c r="J6" s="9" t="inlineStr">
         <is>
-          <t>13:31:04</t>
+          <t>21:08:04</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       <c r="I7" s="11" t="inlineStr"/>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>13:31:14</t>
+          <t>21:08:14</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       <c r="I8" s="9" t="inlineStr"/>
       <c r="J8" s="9" t="inlineStr">
         <is>
-          <t>13:31:23</t>
+          <t>21:08:24</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       <c r="I9" s="11" t="inlineStr"/>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>13:31:40</t>
+          <t>21:08:40</t>
         </is>
       </c>
     </row>
@@ -1381,12 +1381,12 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Login with prabha.testuser@example.com / TestPrabha@9999</t>
+          <t>Login with prabha02102005@gmail.com / 123456789</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>1. Enter prabha.testuser@example.com
+          <t>1. Enter prabha02102005@gmail.com
 2. Enter password
 3. Submit</t>
         </is>
@@ -1411,16 +1411,16 @@
           <t>FAIL may mean account not registered in backend. Body snippet: Smart EV
 ASSISTANT
 P
-Prabha User
-450 Coins
+Prabha
+100 Coins
 Dashboard
 Navigation
-Stations (Chargi</t>
+Stations (Charging St</t>
         </is>
       </c>
       <c r="J10" s="9" t="inlineStr">
         <is>
-          <t>13:31:59</t>
+          <t>21:09:00</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       <c r="I11" s="11" t="inlineStr"/>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>13:32:06</t>
+          <t>21:09:07</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
       <c r="I12" s="9" t="inlineStr"/>
       <c r="J12" s="9" t="inlineStr">
         <is>
-          <t>13:32:13</t>
+          <t>21:09:14</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       <c r="I13" s="11" t="inlineStr"/>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>13:32:20</t>
+          <t>21:09:21</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
       <c r="I14" s="9" t="inlineStr"/>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>13:32:33</t>
+          <t>21:09:33</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
       <c r="I15" s="11" t="inlineStr"/>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>13:32:40</t>
+          <t>21:09:40</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       <c r="I16" s="9" t="inlineStr"/>
       <c r="J16" s="9" t="inlineStr">
         <is>
-          <t>13:32:48</t>
+          <t>21:09:48</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       <c r="I17" s="11" t="inlineStr"/>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>13:32:56</t>
+          <t>21:09:56</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
       <c r="I18" s="9" t="inlineStr"/>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>13:33:08</t>
+          <t>21:10:08</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>URL=http://localhost:3000/dashboard, body_len=1495</t>
+          <t>URL=http://localhost:3000/dashboard, body_len=1493</t>
         </is>
       </c>
       <c r="H19" s="10" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>13:33:28</t>
+          <t>21:10:28</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="I20" s="9" t="inlineStr"/>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>13:33:44</t>
+          <t>21:10:44</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       <c r="I21" s="11" t="inlineStr"/>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>13:33:58</t>
+          <t>21:10:58</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       <c r="I22" s="9" t="inlineStr"/>
       <c r="J22" s="9" t="inlineStr">
         <is>
-          <t>13:34:13</t>
+          <t>21:11:13</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       <c r="I23" s="11" t="inlineStr"/>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>13:34:27</t>
+          <t>21:11:27</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2110,7 @@
       <c r="I24" s="9" t="inlineStr"/>
       <c r="J24" s="9" t="inlineStr">
         <is>
-          <t>13:34:41</t>
+          <t>21:11:41</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2159,7 @@
       <c r="I25" s="11" t="inlineStr"/>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>13:34:55</t>
+          <t>21:11:55</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       <c r="I26" s="9" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr">
         <is>
-          <t>13:35:03</t>
+          <t>21:12:04</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       <c r="I27" s="11" t="inlineStr"/>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>13:35:18</t>
+          <t>21:12:18</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       <c r="I28" s="9" t="inlineStr"/>
       <c r="J28" s="9" t="inlineStr">
         <is>
-          <t>13:35:32</t>
+          <t>21:12:32</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=986</t>
+          <t>URL OK=True, body_len=2194</t>
         </is>
       </c>
       <c r="H29" s="10" t="inlineStr">
@@ -2354,7 +2354,7 @@
       <c r="I29" s="11" t="inlineStr"/>
       <c r="J29" s="11" t="inlineStr">
         <is>
-          <t>13:35:40</t>
+          <t>21:12:40</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2403,7 @@
       <c r="I30" s="9" t="inlineStr"/>
       <c r="J30" s="9" t="inlineStr">
         <is>
-          <t>13:35:48</t>
+          <t>21:12:49</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>13:35:59</t>
+          <t>21:12:59</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       <c r="I32" s="9" t="inlineStr"/>
       <c r="J32" s="9" t="inlineStr">
         <is>
-          <t>13:36:23</t>
+          <t>21:13:23</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
       <c r="I33" s="11" t="inlineStr"/>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>13:36:31</t>
+          <t>21:13:31</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       <c r="I34" s="9" t="inlineStr"/>
       <c r="J34" s="9" t="inlineStr">
         <is>
-          <t>13:36:45</t>
+          <t>21:13:45</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       <c r="I35" s="11" t="inlineStr"/>
       <c r="J35" s="11" t="inlineStr">
         <is>
-          <t>13:36:54</t>
+          <t>21:13:54</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=1533</t>
+          <t>URL OK=True, body_len=1599</t>
         </is>
       </c>
       <c r="H36" s="10" t="inlineStr">
@@ -2699,7 +2699,7 @@
       <c r="I36" s="9" t="inlineStr"/>
       <c r="J36" s="9" t="inlineStr">
         <is>
-          <t>13:37:02</t>
+          <t>21:14:02</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       <c r="I37" s="11" t="inlineStr"/>
       <c r="J37" s="11" t="inlineStr">
         <is>
-          <t>13:37:16</t>
+          <t>21:14:16</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       <c r="I38" s="9" t="inlineStr"/>
       <c r="J38" s="9" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>21:14:24</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
       <c r="I39" s="11" t="inlineStr"/>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>13:37:33</t>
+          <t>21:14:33</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       <c r="I40" s="9" t="inlineStr"/>
       <c r="J40" s="9" t="inlineStr">
         <is>
-          <t>13:37:48</t>
+          <t>21:14:47</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2943,7 @@
       <c r="I41" s="11" t="inlineStr"/>
       <c r="J41" s="11" t="inlineStr">
         <is>
-          <t>13:37:56</t>
+          <t>21:14:55</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=1095</t>
+          <t>URL OK=True, body_len=1247</t>
         </is>
       </c>
       <c r="H42" s="10" t="inlineStr">
@@ -2991,7 +2991,7 @@
       <c r="I42" s="9" t="inlineStr"/>
       <c r="J42" s="9" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>21:15:04</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       <c r="I43" s="11" t="inlineStr"/>
       <c r="J43" s="11" t="inlineStr">
         <is>
-          <t>13:38:18</t>
+          <t>21:15:18</t>
         </is>
       </c>
     </row>
@@ -3077,7 +3077,7 @@
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=1039</t>
+          <t>URL OK=True, body_len=6540</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
@@ -3088,7 +3088,7 @@
       <c r="I44" s="9" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>13:38:27</t>
+          <t>21:15:26</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       <c r="I45" s="11" t="inlineStr"/>
       <c r="J45" s="11" t="inlineStr">
         <is>
-          <t>13:38:41</t>
+          <t>21:15:40</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3185,7 @@
       <c r="I46" s="9" t="inlineStr"/>
       <c r="J46" s="9" t="inlineStr">
         <is>
-          <t>13:38:49</t>
+          <t>21:15:49</t>
         </is>
       </c>
     </row>
@@ -3234,7 +3234,7 @@
       <c r="I47" s="11" t="inlineStr"/>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>13:39:03</t>
+          <t>21:16:03</t>
         </is>
       </c>
     </row>
@@ -3282,7 +3282,7 @@
       <c r="I48" s="9" t="inlineStr"/>
       <c r="J48" s="9" t="inlineStr">
         <is>
-          <t>13:39:11</t>
+          <t>21:16:11</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       <c r="I49" s="11" t="inlineStr"/>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>13:39:26</t>
+          <t>21:16:25</t>
         </is>
       </c>
     </row>
@@ -3380,7 +3380,7 @@
       <c r="I50" s="9" t="inlineStr"/>
       <c r="J50" s="9" t="inlineStr">
         <is>
-          <t>13:39:34</t>
+          <t>21:16:34</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3428,7 @@
       <c r="I51" s="11" t="inlineStr"/>
       <c r="J51" s="11" t="inlineStr">
         <is>
-          <t>13:39:42</t>
+          <t>21:16:42</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       <c r="I52" s="9" t="inlineStr"/>
       <c r="J52" s="9" t="inlineStr">
         <is>
-          <t>13:39:56</t>
+          <t>21:16:56</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="G53" s="11" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=2788</t>
+          <t>URL OK=True, body_len=3029</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
@@ -3525,7 +3525,7 @@
       <c r="I53" s="11" t="inlineStr"/>
       <c r="J53" s="11" t="inlineStr">
         <is>
-          <t>13:40:05</t>
+          <t>21:17:05</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       <c r="I54" s="9" t="inlineStr"/>
       <c r="J54" s="9" t="inlineStr">
         <is>
-          <t>13:40:19</t>
+          <t>21:17:19</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
       <c r="I55" s="11" t="inlineStr"/>
       <c r="J55" s="11" t="inlineStr">
         <is>
-          <t>13:40:27</t>
+          <t>21:17:27</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       <c r="I56" s="9" t="inlineStr"/>
       <c r="J56" s="9" t="inlineStr">
         <is>
-          <t>13:40:41</t>
+          <t>21:17:41</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3720,7 @@
       <c r="I57" s="11" t="inlineStr"/>
       <c r="J57" s="11" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>21:17:50</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       <c r="I58" s="9" t="inlineStr"/>
       <c r="J58" s="9" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>21:17:50</t>
         </is>
       </c>
     </row>
@@ -3817,7 +3817,7 @@
       <c r="I59" s="11" t="inlineStr"/>
       <c r="J59" s="11" t="inlineStr">
         <is>
-          <t>13:40:56</t>
+          <t>21:17:56</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3866,7 @@
       <c r="I60" s="9" t="inlineStr"/>
       <c r="J60" s="9" t="inlineStr">
         <is>
-          <t>13:41:11</t>
+          <t>21:18:11</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       <c r="I61" s="11" t="inlineStr"/>
       <c r="J61" s="11" t="inlineStr">
         <is>
-          <t>13:41:19</t>
+          <t>21:18:19</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       <c r="I62" s="9" t="inlineStr"/>
       <c r="J62" s="9" t="inlineStr">
         <is>
-          <t>13:41:27</t>
+          <t>21:18:27</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
       <c r="I63" s="11" t="inlineStr"/>
       <c r="J63" s="11" t="inlineStr">
         <is>
-          <t>13:41:41</t>
+          <t>21:18:41</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="J64" s="9" t="inlineStr">
         <is>
-          <t>13:42:06</t>
+          <t>21:19:07</t>
         </is>
       </c>
     </row>
@@ -4143,13 +4143,13 @@
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
-          <t>html_len=93765</t>
+          <t>html_len=93759</t>
         </is>
       </c>
       <c r="E2" s="13" t="inlineStr"/>
       <c r="F2" s="13" t="inlineStr">
         <is>
-          <t>13:30:40</t>
+          <t>21:07:41</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4177,7 @@
       <c r="E3" s="13" t="inlineStr"/>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>13:30:43</t>
+          <t>21:07:44</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       <c r="E4" s="13" t="inlineStr"/>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t>13:30:49</t>
+          <t>21:07:50</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4233,7 @@
       <c r="E5" s="13" t="inlineStr"/>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>13:30:56</t>
+          <t>21:07:56</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       <c r="E6" s="13" t="inlineStr"/>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>13:31:04</t>
+          <t>21:08:04</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
       <c r="E7" s="13" t="inlineStr"/>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>13:31:14</t>
+          <t>21:08:14</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4317,7 @@
       <c r="E8" s="13" t="inlineStr"/>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>13:31:23</t>
+          <t>21:08:24</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4345,7 @@
       <c r="E9" s="13" t="inlineStr"/>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>13:31:40</t>
+          <t>21:08:40</t>
         </is>
       </c>
     </row>
@@ -4375,16 +4375,16 @@
           <t>FAIL may mean account not registered in backend. Body snippet: Smart EV
 ASSISTANT
 P
-Prabha User
-450 Coins
+Prabha
+100 Coins
 Dashboard
 Navigation
-Stations (Chargi</t>
+Stations (Charging St</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>13:31:59</t>
+          <t>21:09:00</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4412,7 @@
       <c r="E11" s="13" t="inlineStr"/>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>13:32:06</t>
+          <t>21:09:07</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       <c r="E12" s="13" t="inlineStr"/>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>13:32:13</t>
+          <t>21:09:14</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4468,7 @@
       <c r="E13" s="13" t="inlineStr"/>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>13:32:20</t>
+          <t>21:09:21</t>
         </is>
       </c>
     </row>
@@ -4496,7 +4496,7 @@
       <c r="E14" s="13" t="inlineStr"/>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>13:32:33</t>
+          <t>21:09:33</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       <c r="E15" s="13" t="inlineStr"/>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>13:32:40</t>
+          <t>21:09:40</t>
         </is>
       </c>
     </row>
@@ -4552,7 +4552,7 @@
       <c r="E16" s="13" t="inlineStr"/>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>13:32:48</t>
+          <t>21:09:48</t>
         </is>
       </c>
     </row>
@@ -4580,7 +4580,7 @@
       <c r="E17" s="13" t="inlineStr"/>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>13:32:56</t>
+          <t>21:09:56</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       <c r="E18" s="13" t="inlineStr"/>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>13:33:08</t>
+          <t>21:10:08</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>URL=http://localhost:3000/dashboard, body_len=1495</t>
+          <t>URL=http://localhost:3000/dashboard, body_len=1493</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -4640,7 +4640,7 @@
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>13:33:28</t>
+          <t>21:10:28</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       <c r="E20" s="13" t="inlineStr"/>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>13:33:44</t>
+          <t>21:10:44</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4696,7 @@
       <c r="E21" s="13" t="inlineStr"/>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>13:33:58</t>
+          <t>21:10:58</t>
         </is>
       </c>
     </row>
@@ -4724,7 +4724,7 @@
       <c r="E22" s="13" t="inlineStr"/>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>13:34:13</t>
+          <t>21:11:13</t>
         </is>
       </c>
     </row>
@@ -4752,7 +4752,7 @@
       <c r="E23" s="13" t="inlineStr"/>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>13:34:27</t>
+          <t>21:11:27</t>
         </is>
       </c>
     </row>
@@ -4780,7 +4780,7 @@
       <c r="E24" s="13" t="inlineStr"/>
       <c r="F24" s="13" t="inlineStr">
         <is>
-          <t>13:34:41</t>
+          <t>21:11:41</t>
         </is>
       </c>
     </row>
@@ -4808,7 +4808,7 @@
       <c r="E25" s="13" t="inlineStr"/>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>13:34:55</t>
+          <t>21:11:55</t>
         </is>
       </c>
     </row>
@@ -4836,7 +4836,7 @@
       <c r="E26" s="13" t="inlineStr"/>
       <c r="F26" s="13" t="inlineStr">
         <is>
-          <t>13:35:03</t>
+          <t>21:12:04</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       <c r="E27" s="13" t="inlineStr"/>
       <c r="F27" s="13" t="inlineStr">
         <is>
-          <t>13:35:18</t>
+          <t>21:12:18</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
       <c r="E28" s="13" t="inlineStr"/>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>13:35:32</t>
+          <t>21:12:32</t>
         </is>
       </c>
     </row>
@@ -4914,13 +4914,13 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=986</t>
+          <t>URL OK=True, body_len=2194</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr"/>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>13:35:40</t>
+          <t>21:12:40</t>
         </is>
       </c>
     </row>
@@ -4948,7 +4948,7 @@
       <c r="E30" s="13" t="inlineStr"/>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>13:35:48</t>
+          <t>21:12:49</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
-          <t>13:35:59</t>
+          <t>21:12:59</t>
         </is>
       </c>
     </row>
@@ -5008,7 +5008,7 @@
       <c r="E32" s="13" t="inlineStr"/>
       <c r="F32" s="13" t="inlineStr">
         <is>
-          <t>13:36:23</t>
+          <t>21:13:23</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
       <c r="E33" s="13" t="inlineStr"/>
       <c r="F33" s="13" t="inlineStr">
         <is>
-          <t>13:36:31</t>
+          <t>21:13:31</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       <c r="E34" s="13" t="inlineStr"/>
       <c r="F34" s="13" t="inlineStr">
         <is>
-          <t>13:36:45</t>
+          <t>21:13:45</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5092,7 @@
       <c r="E35" s="13" t="inlineStr"/>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>13:36:54</t>
+          <t>21:13:54</t>
         </is>
       </c>
     </row>
@@ -5114,13 +5114,13 @@
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=1533</t>
+          <t>URL OK=True, body_len=1599</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr"/>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>13:37:02</t>
+          <t>21:14:02</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       <c r="E37" s="13" t="inlineStr"/>
       <c r="F37" s="13" t="inlineStr">
         <is>
-          <t>13:37:16</t>
+          <t>21:14:16</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       <c r="E38" s="13" t="inlineStr"/>
       <c r="F38" s="13" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>21:14:24</t>
         </is>
       </c>
     </row>
@@ -5204,7 +5204,7 @@
       <c r="E39" s="13" t="inlineStr"/>
       <c r="F39" s="13" t="inlineStr">
         <is>
-          <t>13:37:33</t>
+          <t>21:14:33</t>
         </is>
       </c>
     </row>
@@ -5232,7 +5232,7 @@
       <c r="E40" s="13" t="inlineStr"/>
       <c r="F40" s="13" t="inlineStr">
         <is>
-          <t>13:37:48</t>
+          <t>21:14:47</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5260,7 @@
       <c r="E41" s="13" t="inlineStr"/>
       <c r="F41" s="13" t="inlineStr">
         <is>
-          <t>13:37:56</t>
+          <t>21:14:55</t>
         </is>
       </c>
     </row>
@@ -5282,13 +5282,13 @@
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=1095</t>
+          <t>URL OK=True, body_len=1247</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr"/>
       <c r="F42" s="13" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>21:15:04</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       <c r="E43" s="13" t="inlineStr"/>
       <c r="F43" s="13" t="inlineStr">
         <is>
-          <t>13:38:18</t>
+          <t>21:15:18</t>
         </is>
       </c>
     </row>
@@ -5338,13 +5338,13 @@
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=1039</t>
+          <t>URL OK=True, body_len=6540</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr"/>
       <c r="F44" s="13" t="inlineStr">
         <is>
-          <t>13:38:27</t>
+          <t>21:15:26</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5372,7 @@
       <c r="E45" s="13" t="inlineStr"/>
       <c r="F45" s="13" t="inlineStr">
         <is>
-          <t>13:38:41</t>
+          <t>21:15:40</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
       <c r="E46" s="13" t="inlineStr"/>
       <c r="F46" s="13" t="inlineStr">
         <is>
-          <t>13:38:49</t>
+          <t>21:15:49</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       <c r="E47" s="13" t="inlineStr"/>
       <c r="F47" s="13" t="inlineStr">
         <is>
-          <t>13:39:03</t>
+          <t>21:16:03</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       <c r="E48" s="13" t="inlineStr"/>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>13:39:11</t>
+          <t>21:16:11</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       <c r="E49" s="13" t="inlineStr"/>
       <c r="F49" s="13" t="inlineStr">
         <is>
-          <t>13:39:26</t>
+          <t>21:16:25</t>
         </is>
       </c>
     </row>
@@ -5512,7 +5512,7 @@
       <c r="E50" s="13" t="inlineStr"/>
       <c r="F50" s="13" t="inlineStr">
         <is>
-          <t>13:39:34</t>
+          <t>21:16:34</t>
         </is>
       </c>
     </row>
@@ -5540,7 +5540,7 @@
       <c r="E51" s="13" t="inlineStr"/>
       <c r="F51" s="13" t="inlineStr">
         <is>
-          <t>13:39:42</t>
+          <t>21:16:42</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       <c r="E52" s="13" t="inlineStr"/>
       <c r="F52" s="13" t="inlineStr">
         <is>
-          <t>13:39:56</t>
+          <t>21:16:56</t>
         </is>
       </c>
     </row>
@@ -5590,13 +5590,13 @@
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>URL OK=True, body_len=2788</t>
+          <t>URL OK=True, body_len=3029</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr"/>
       <c r="F53" s="13" t="inlineStr">
         <is>
-          <t>13:40:05</t>
+          <t>21:17:05</t>
         </is>
       </c>
     </row>
@@ -5624,7 +5624,7 @@
       <c r="E54" s="13" t="inlineStr"/>
       <c r="F54" s="13" t="inlineStr">
         <is>
-          <t>13:40:19</t>
+          <t>21:17:19</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5652,7 @@
       <c r="E55" s="13" t="inlineStr"/>
       <c r="F55" s="13" t="inlineStr">
         <is>
-          <t>13:40:27</t>
+          <t>21:17:27</t>
         </is>
       </c>
     </row>
@@ -5680,7 +5680,7 @@
       <c r="E56" s="13" t="inlineStr"/>
       <c r="F56" s="13" t="inlineStr">
         <is>
-          <t>13:40:41</t>
+          <t>21:17:41</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       <c r="E57" s="13" t="inlineStr"/>
       <c r="F57" s="13" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>21:17:50</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5736,7 @@
       <c r="E58" s="13" t="inlineStr"/>
       <c r="F58" s="13" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>21:17:50</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
       <c r="E59" s="13" t="inlineStr"/>
       <c r="F59" s="13" t="inlineStr">
         <is>
-          <t>13:40:56</t>
+          <t>21:17:56</t>
         </is>
       </c>
     </row>
@@ -5792,7 +5792,7 @@
       <c r="E60" s="13" t="inlineStr"/>
       <c r="F60" s="13" t="inlineStr">
         <is>
-          <t>13:41:11</t>
+          <t>21:18:11</t>
         </is>
       </c>
     </row>
@@ -5820,7 +5820,7 @@
       <c r="E61" s="13" t="inlineStr"/>
       <c r="F61" s="13" t="inlineStr">
         <is>
-          <t>13:41:19</t>
+          <t>21:18:19</t>
         </is>
       </c>
     </row>
@@ -5848,7 +5848,7 @@
       <c r="E62" s="13" t="inlineStr"/>
       <c r="F62" s="13" t="inlineStr">
         <is>
-          <t>13:41:27</t>
+          <t>21:18:27</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
       <c r="E63" s="13" t="inlineStr"/>
       <c r="F63" s="13" t="inlineStr">
         <is>
-          <t>13:41:41</t>
+          <t>21:18:41</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="F64" s="13" t="inlineStr">
         <is>
-          <t>13:42:06</t>
+          <t>21:19:07</t>
         </is>
       </c>
     </row>

</xml_diff>